<commit_message>
Added 7 day work chart
</commit_message>
<xml_diff>
--- a/data/manpower_resources.xlsx
+++ b/data/manpower_resources.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Machine Status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Manpower Status" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Manhour Status" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machine Status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manpower Status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manhour Status" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -513,7 +513,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>13-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -522,13 +522,13 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>16-Jun-2026</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -537,13 +537,13 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -552,13 +552,13 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -567,13 +567,13 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -582,13 +582,13 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>20-Jun-2026</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -597,13 +597,13 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>21-Jun-2026</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -611,14 +611,12 @@
           <t>Hammer</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
-        <v>2</v>
-      </c>
+      <c r="C9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>20-Jun-2026</t>
+          <t>22-Jun-2026</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -633,7 +631,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>21-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -641,12 +639,14 @@
           <t>Hammer</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
+      <c r="C11" s="7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>22-Jun-2026</t>
+          <t>24-Jun-2026</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>25-Jun-2026</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>26-Jun-2026</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>29-Jun-2026</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -736,7 +736,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -745,13 +745,13 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -790,7 +790,22 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>13-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -804,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -826,17 +841,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>13-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
@@ -846,37 +861,37 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>16-Jun-2026</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -886,37 +901,37 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>20-Jun-2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>22-Jun-2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>20-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>22-Jun-2026</t>
+          <t>24-Jun-2026</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -926,7 +941,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>25-Jun-2026</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -936,7 +951,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>26-Jun-2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -946,71 +961,81 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>29-Jun-2026</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>13-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1024,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1071,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>12-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -1056,7 +1081,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>13-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
@@ -1066,7 +1091,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>16-Jun-2026</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1076,7 +1101,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -1086,7 +1111,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -1096,7 +1121,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -1106,7 +1131,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>20-Jun-2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -1116,7 +1141,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>22-Jun-2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
@@ -1126,7 +1151,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>20-Jun-2026</t>
+          <t>23-Jun-2026</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -1136,7 +1161,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>22-Jun-2026</t>
+          <t>24-Jun-2026</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -1146,7 +1171,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>25-Jun-2026</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -1156,7 +1181,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>26-Jun-2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -1166,7 +1191,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>29-Jun-2026</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -1176,7 +1201,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
@@ -1186,7 +1211,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -1196,7 +1221,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
@@ -1206,7 +1231,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -1216,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -1226,10 +1251,20 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>13-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add initial implementation of Sheet Pile Installation Planner in __probe.html
- Created a new HTML file for the Sheet Pile Installation Planner application.
- Included necessary meta tags, stylesheets, and scripts for functionality.
- Structured the layout with a header, home module picker, and main planner interface.
- Implemented sections for data file uploads, plan parameters, results display, and validation.
- Added interactive elements for user input and data visualization.
</commit_message>
<xml_diff>
--- a/data/manpower_resources.xlsx
+++ b/data/manpower_resources.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -522,13 +522,13 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -543,7 +543,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -552,13 +552,13 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -582,13 +582,13 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>13-Jul-2026</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -597,13 +597,13 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -618,7 +618,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -627,13 +627,13 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>10-Jul-2026</t>
+          <t>17-Jul-2026</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>12-Jul-2026</t>
+          <t>18-Jul-2026</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>13-Jul-2026</t>
+          <t>19-Jul-2026</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -672,13 +672,13 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>20-Jul-2026</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -687,13 +687,13 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>15-Jul-2026</t>
+          <t>21-Jul-2026</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>17-Jul-2026</t>
+          <t>22-Jul-2026</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -717,13 +717,13 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>18-Jul-2026</t>
+          <t>23-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -732,13 +732,13 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>19-Jul-2026</t>
+          <t>24-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -747,13 +747,13 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>20-Jul-2026</t>
+          <t>25-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -762,13 +762,13 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-2026</t>
+          <t>26-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -777,7 +777,37 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>27-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>28-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -791,7 +821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -813,191 +843,211 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>13-Jul-2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>10-Jul-2026</t>
+          <t>17-Jul-2026</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>12-Jul-2026</t>
+          <t>18-Jul-2026</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>13-Jul-2026</t>
+          <t>19-Jul-2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>20-Jul-2026</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>15-Jul-2026</t>
+          <t>21-Jul-2026</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>17-Jul-2026</t>
+          <t>22-Jul-2026</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>18-Jul-2026</t>
+          <t>23-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>19-Jul-2026</t>
+          <t>24-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>20-Jul-2026</t>
+          <t>25-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-2026</t>
+          <t>26-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>39</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>27-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>28-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1011,7 +1061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1033,7 +1083,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -1043,7 +1093,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>24-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
@@ -1053,7 +1103,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>25-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1063,7 +1113,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>26-Jun-2026</t>
+          <t>03-Jul-2026</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -1073,7 +1123,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>29-Jun-2026</t>
+          <t>10-Jul-2026</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -1083,7 +1133,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>12-Jul-2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -1093,7 +1143,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>13-Jul-2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -1103,7 +1153,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
@@ -1113,7 +1163,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>03-Jul-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -1123,7 +1173,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>10-Jul-2026</t>
+          <t>17-Jul-2026</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -1133,7 +1183,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>12-Jul-2026</t>
+          <t>18-Jul-2026</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -1143,7 +1193,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>13-Jul-2026</t>
+          <t>19-Jul-2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -1153,7 +1203,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>20-Jul-2026</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -1163,7 +1213,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>15-Jul-2026</t>
+          <t>21-Jul-2026</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
@@ -1173,7 +1223,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>17-Jul-2026</t>
+          <t>22-Jul-2026</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -1183,7 +1233,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>18-Jul-2026</t>
+          <t>23-Jul-2026</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
@@ -1193,7 +1243,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>19-Jul-2026</t>
+          <t>24-Jul-2026</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -1203,7 +1253,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>20-Jul-2026</t>
+          <t>25-Jul-2026</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -1213,10 +1263,30 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>21-Jul-2026</t>
+          <t>26-Jul-2026</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>27-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>28-Jul-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>